<commit_message>
Update input data file paths, enhance initial solution logic, and add feasibility testing template
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/inputData/Parameters.xlsx
+++ b/inputData/Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/inputData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5EA3A5C-B68C-8444-868C-6B4E1B007986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6BECB4-727C-4CD8-864E-4DD0622BE9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="11920" windowHeight="16340" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="9" r:id="rId1"/>
@@ -156,6 +156,9 @@
     <t>fd_sum</t>
   </si>
   <si>
+    <t>2,1% battery charged per unit time</t>
+  </si>
+  <si>
     <t>rt_{i,j} = 0.2 min/km</t>
   </si>
   <si>
@@ -168,6 +171,9 @@
     <t>penalty for not serving passengergroup</t>
   </si>
   <si>
+    <t>penalty for exceeding bmax</t>
+  </si>
+  <si>
     <t>bmid</t>
   </si>
   <si>
@@ -178,12 +184,6 @@
   </si>
   <si>
     <t>minuts/unit</t>
-  </si>
-  <si>
-    <t>penalty for exceeding bmid</t>
-  </si>
-  <si>
-    <t>2,1% battery charged per min</t>
   </si>
 </sst>
 </file>
@@ -607,18 +607,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15C49E0-A7B4-734A-8962-DC2A879F4079}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.6640625" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -629,7 +629,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -640,18 +640,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B4" s="4">
         <v>400</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -659,10 +659,10 @@
         <v>300</v>
       </c>
       <c r="D5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -673,7 +673,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -684,7 +684,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -693,10 +693,10 @@
         <v>0.2</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -707,7 +707,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -718,9 +718,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B11" s="4">
         <v>80</v>
@@ -729,7 +729,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -740,18 +740,18 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13" s="4">
         <v>20</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -760,10 +760,10 @@
         <v>2.11</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -775,7 +775,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -787,7 +787,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -799,15 +799,15 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B20" s="4">
         <v>1</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -819,7 +819,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF0D5EA-53B5-1240-9D84-6FE223856A18}">
   <dimension ref="A1:N24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -828,7 +828,7 @@
     <col min="6" max="6" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A1" s="12" t="s">
         <v>36</v>
       </c>
@@ -867,7 +867,7 @@
       </c>
       <c r="N1" s="6"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -915,7 +915,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>1</v>
       </c>
@@ -963,7 +963,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1056,7 +1056,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>2</v>
       </c>
@@ -1095,7 +1095,7 @@
         <v>2489</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>2</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>2109</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1173,7 +1173,7 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1211,7 +1211,7 @@
         <v>1915.6666666666665</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>3</v>
       </c>
@@ -1249,7 +1249,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>4</v>
       </c>
@@ -1287,7 +1287,7 @@
         <v>1767</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>1</v>
       </c>
@@ -1303,7 +1303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>3</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>4</v>
       </c>
@@ -1341,7 +1341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>5</v>
       </c>
@@ -1353,19 +1353,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="5:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="5:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="5:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="5:5" x14ac:dyDescent="0.4">
       <c r="E24" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update input data files and adjust parameters for heuristic algorithm
- Changed the input Excel file from `inputData.xlsx` to `inputDataMicro.xlsx` for testing purposes.
- Updated the maximum time parameter from 60 to 10 in the heuristic function call to reduce computation time.
- Modified the `Parameters.xlsx` file to reflect necessary changes.
- Added a new `inputDataMicro.xlsx` file to the input data directory.

Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/inputData/Parameters.xlsx
+++ b/inputData/Parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6BECB4-727C-4CD8-864E-4DD0622BE9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E853C988-B6AC-4B4D-A660-2EEFA7D08239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
@@ -656,7 +656,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="4">
-        <v>300</v>
+        <v>3000</v>
       </c>
       <c r="D5" t="s">
         <v>43</v>
@@ -689,8 +689,7 @@
         <v>19</v>
       </c>
       <c r="B8" s="4">
-        <f>0.2/B20</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D8" t="s">
         <v>40</v>
@@ -734,7 +733,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="4">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update Parameters.xlsx with new input data
</commit_message>
<xml_diff>
--- a/inputData/Parameters.xlsx
+++ b/inputData/Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E853C988-B6AC-4B4D-A660-2EEFA7D08239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A24315D7-801C-405F-93C4-E43B62ED5969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="9" r:id="rId1"/>
@@ -656,7 +656,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="4">
-        <v>3000</v>
+        <v>300</v>
       </c>
       <c r="D5" t="s">
         <v>43</v>

</xml_diff>

<commit_message>
Increased entime to 8 hours
</commit_message>
<xml_diff>
--- a/inputData/Parameters.xlsx
+++ b/inputData/Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/inputData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC525445-B921-7444-8BE9-F0D2537C0186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CBE765F-9084-4140-9ADF-71B92BC0CEA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16320" activeTab="1" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="9" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="61">
   <si>
     <t>cap_u</t>
   </si>
@@ -647,19 +647,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15C49E0-A7B4-734A-8962-DC2A879F4079}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.6640625" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:4" dyDescent="0.2">
-      <c r="A2" t="s" s="1">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="4">
@@ -669,7 +669,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -680,7 +680,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -691,7 +691,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:4" dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -702,7 +702,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:4" dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -713,7 +713,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -724,7 +724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -736,7 +736,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:4" dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -747,7 +747,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -758,7 +758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>45</v>
       </c>
@@ -769,7 +769,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="12" spans="1:4" dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -780,18 +780,18 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="13" spans="1:4" dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>42</v>
       </c>
       <c r="B13" s="4">
         <v>20</v>
       </c>
-      <c r="D13" t="s" s="3">
+      <c r="D13" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:4" dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -799,11 +799,11 @@
         <f>2.11*B20</f>
         <v>2.11</v>
       </c>
-      <c r="D14" t="s" s="3">
+      <c r="D14" s="3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:4" dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -811,11 +811,11 @@
         <f>30/B20</f>
         <v>30</v>
       </c>
-      <c r="D15" t="s" s="3">
+      <c r="D15" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:4" dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -823,30 +823,29 @@
         <f>20/B20</f>
         <v>20</v>
       </c>
-      <c r="D16" t="s" s="3">
+      <c r="D16" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:4" dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>6</v>
       </c>
       <c r="B17" s="4">
-        <f>120/B20</f>
-        <v>120</v>
-      </c>
-      <c r="D17" t="s" s="3">
+        <v>780</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:4" dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>41</v>
       </c>
       <c r="B20" s="4">
         <v>1</v>
       </c>
-      <c r="D20" t="s" s="3">
+      <c r="D20" s="3" t="s">
         <v>48</v>
       </c>
     </row>
@@ -859,7 +858,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF0D5EA-53B5-1240-9D84-6FE223856A18}">
   <dimension ref="A1:P59"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="17.1640625" customWidth="1"/>
@@ -869,44 +868,44 @@
     <col min="8" max="8" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" dyDescent="0.2">
-      <c r="A1" t="s" s="9">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A1" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B1" t="s" s="5">
+      <c r="B1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C1" t="s" s="5">
+      <c r="C1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D1" t="s" s="5">
+      <c r="D1" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E1" t="s" s="5">
+      <c r="E1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F1" t="s" s="5">
+      <c r="F1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G1" t="s" s="5">
+      <c r="G1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="H1" t="s" s="5">
+      <c r="H1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="I1" t="s" s="5">
+      <c r="I1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="J1" t="s" s="5">
+      <c r="J1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="K1" t="s" s="5">
+      <c r="K1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="L1" t="s" s="5">
+      <c r="L1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s" s="6">
+      <c r="N1" s="6" t="s">
         <v>19</v>
       </c>
       <c r="O1" s="7">
@@ -914,24 +913,24 @@
       </c>
       <c r="P1" s="6"/>
     </row>
-    <row r="2" spans="1:16" dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="8">
         <v>2</v>
       </c>
-      <c r="C2" t="s" s="1">
+      <c r="C2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D2" t="s" s="2">
+      <c r="D2" s="2" t="s">
         <v>52</v>
       </c>
       <c r="E2">
-        <v>185.0</v>
+        <v>185</v>
       </c>
       <c r="F2">
-        <v>219.0</v>
+        <v>219</v>
       </c>
       <c r="G2">
         <v>43.8</v>
@@ -940,16 +939,16 @@
         <v>4.2</v>
       </c>
       <c r="I2">
-        <v>4161.0</v>
+        <v>4161</v>
       </c>
       <c r="J2">
-        <v>1647.0</v>
+        <v>1647</v>
       </c>
       <c r="K2">
-        <v>5808.0</v>
+        <v>5808</v>
       </c>
       <c r="L2">
-        <v>4161.0</v>
+        <v>4161</v>
       </c>
       <c r="N2" t="s">
         <v>29</v>
@@ -961,42 +960,42 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:16" dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" s="8">
         <v>3</v>
       </c>
-      <c r="C3" t="s" s="1">
+      <c r="C3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D3" t="s" s="2">
+      <c r="D3" s="2" t="s">
         <v>53</v>
       </c>
       <c r="E3">
-        <v>82.0</v>
+        <v>82</v>
       </c>
       <c r="F3">
-        <v>88.0</v>
+        <v>88</v>
       </c>
       <c r="G3">
-        <v>17.6</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="H3">
         <v>4.7</v>
       </c>
       <c r="I3">
-        <v>1672.0</v>
+        <v>1672</v>
       </c>
       <c r="J3">
-        <v>751.0</v>
+        <v>751</v>
       </c>
       <c r="K3">
-        <v>2423.0</v>
+        <v>2423</v>
       </c>
       <c r="L3">
-        <v>1672.0</v>
+        <v>1672</v>
       </c>
       <c r="N3" t="s">
         <v>31</v>
@@ -1009,24 +1008,24 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:16" dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" s="8">
         <v>4</v>
       </c>
-      <c r="C4" t="s" s="1">
+      <c r="C4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D4" t="s" s="1">
+      <c r="D4" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E4">
-        <v>228.0</v>
+        <v>228</v>
       </c>
       <c r="F4">
-        <v>147.0</v>
+        <v>147</v>
       </c>
       <c r="G4">
         <v>29.4</v>
@@ -1035,16 +1034,16 @@
         <v>7.8</v>
       </c>
       <c r="I4">
-        <v>2793.0</v>
+        <v>2793</v>
       </c>
       <c r="J4">
-        <v>2317.0</v>
+        <v>2317</v>
       </c>
       <c r="K4">
-        <v>5110.0</v>
+        <v>5110</v>
       </c>
       <c r="L4">
-        <v>2793.0</v>
+        <v>2793</v>
       </c>
       <c r="N4" t="s">
         <v>33</v>
@@ -1053,24 +1052,24 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="5" spans="1:16" dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" s="8">
         <v>5</v>
       </c>
-      <c r="C5" t="s" s="1">
+      <c r="C5" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D5" t="s" s="1">
+      <c r="D5" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E5">
-        <v>126.0</v>
+        <v>126</v>
       </c>
       <c r="F5">
-        <v>147.0</v>
+        <v>147</v>
       </c>
       <c r="G5">
         <v>29.4</v>
@@ -1079,16 +1078,16 @@
         <v>4.3</v>
       </c>
       <c r="I5">
-        <v>2793.0</v>
+        <v>2793</v>
       </c>
       <c r="J5">
-        <v>1127.0</v>
+        <v>1127</v>
       </c>
       <c r="K5">
-        <v>3920.0</v>
+        <v>3920</v>
       </c>
       <c r="L5">
-        <v>2793.0</v>
+        <v>2793</v>
       </c>
       <c r="N5" t="s">
         <v>34</v>
@@ -1100,24 +1099,24 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:16" dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" s="8">
         <v>6</v>
       </c>
-      <c r="C6" t="s" s="1">
+      <c r="C6" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D6" t="s" s="1">
+      <c r="D6" s="1" t="s">
         <v>56</v>
       </c>
       <c r="E6">
-        <v>205.0</v>
+        <v>205</v>
       </c>
       <c r="F6">
-        <v>197.0</v>
+        <v>197</v>
       </c>
       <c r="G6">
         <v>39.4</v>
@@ -1126,37 +1125,37 @@
         <v>5.2</v>
       </c>
       <c r="I6">
-        <v>3743.0</v>
+        <v>3743</v>
       </c>
       <c r="J6">
-        <v>1932.0</v>
+        <v>1932</v>
       </c>
       <c r="K6">
-        <v>5675.0</v>
+        <v>5675</v>
       </c>
       <c r="L6">
-        <v>3743.0</v>
+        <v>3743</v>
       </c>
       <c r="O6" s="4"/>
     </row>
-    <row r="7" spans="1:16" dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7" s="8">
         <v>7</v>
       </c>
-      <c r="C7" t="s" s="1">
+      <c r="C7" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D7" t="s" s="1">
+      <c r="D7" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E7">
-        <v>263.0</v>
+        <v>263</v>
       </c>
       <c r="F7">
-        <v>227.0</v>
+        <v>227</v>
       </c>
       <c r="G7">
         <v>45.4</v>
@@ -1165,154 +1164,154 @@
         <v>5.8</v>
       </c>
       <c r="I7">
-        <v>4313.0</v>
+        <v>4313</v>
       </c>
       <c r="J7">
-        <v>2539.0</v>
+        <v>2539</v>
       </c>
       <c r="K7">
-        <v>6852.0</v>
+        <v>6852</v>
       </c>
       <c r="L7">
-        <v>4313.0</v>
+        <v>4313</v>
       </c>
       <c r="O7" s="4"/>
     </row>
-    <row r="8" spans="1:16" dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" s="8">
         <v>8</v>
       </c>
-      <c r="C8" t="s" s="1">
+      <c r="C8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D8" t="s" s="1">
+      <c r="D8" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E8">
-        <v>143.0</v>
+        <v>143</v>
       </c>
       <c r="F8">
-        <v>184.0</v>
+        <v>184</v>
       </c>
       <c r="G8">
-        <v>36.8</v>
+        <v>36.799999999999997</v>
       </c>
       <c r="H8">
         <v>3.9</v>
       </c>
       <c r="I8">
-        <v>3496.0</v>
+        <v>3496</v>
       </c>
       <c r="J8">
-        <v>1239.0</v>
+        <v>1239</v>
       </c>
       <c r="K8">
-        <v>4735.0</v>
+        <v>4735</v>
       </c>
       <c r="L8">
-        <v>3496.0</v>
+        <v>3496</v>
       </c>
       <c r="O8" s="4"/>
     </row>
-    <row r="9" spans="1:16" dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>1</v>
       </c>
       <c r="B9" s="8">
         <v>9</v>
       </c>
-      <c r="C9" t="s" s="1">
+      <c r="C9" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D9" t="s" s="1">
+      <c r="D9" s="1" t="s">
         <v>59</v>
       </c>
       <c r="E9">
-        <v>155.0</v>
+        <v>155</v>
       </c>
       <c r="F9">
-        <v>193.0</v>
+        <v>193</v>
       </c>
       <c r="G9">
         <v>38.6</v>
       </c>
       <c r="H9">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I9">
-        <v>3667.0</v>
+        <v>3667</v>
       </c>
       <c r="J9">
-        <v>1358.0</v>
+        <v>1358</v>
       </c>
       <c r="K9">
-        <v>5025.0</v>
+        <v>5025</v>
       </c>
       <c r="L9">
-        <v>3667.0</v>
+        <v>3667</v>
       </c>
       <c r="O9" s="4"/>
     </row>
-    <row r="10" spans="1:16" dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>1</v>
       </c>
       <c r="B10" s="8">
         <v>10</v>
       </c>
-      <c r="C10" t="s" s="1">
+      <c r="C10" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D10" t="s" s="1">
+      <c r="D10" s="1" t="s">
         <v>60</v>
       </c>
       <c r="E10">
-        <v>42.0</v>
+        <v>42</v>
       </c>
       <c r="F10">
-        <v>41.0</v>
+        <v>41</v>
       </c>
       <c r="G10">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="H10">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I10">
-        <v>779.0</v>
+        <v>779</v>
       </c>
       <c r="J10">
-        <v>394.0</v>
+        <v>394</v>
       </c>
       <c r="K10">
-        <v>1173.0</v>
+        <v>1173</v>
       </c>
       <c r="L10">
-        <v>779.0</v>
+        <v>779</v>
       </c>
       <c r="O10" s="4"/>
     </row>
-    <row r="11" spans="1:16" dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>2</v>
       </c>
       <c r="B11" s="8">
         <v>3</v>
       </c>
-      <c r="C11" t="s" s="2">
+      <c r="C11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D11" t="s" s="2">
+      <c r="D11" s="2" t="s">
         <v>53</v>
       </c>
       <c r="E11">
-        <v>173.0</v>
+        <v>173</v>
       </c>
       <c r="F11">
-        <v>131.0</v>
+        <v>131</v>
       </c>
       <c r="G11">
         <v>26.2</v>
@@ -1321,226 +1320,226 @@
         <v>6.6</v>
       </c>
       <c r="I11">
-        <v>2489.0</v>
+        <v>2489</v>
       </c>
       <c r="J11">
-        <v>1713.0</v>
+        <v>1713</v>
       </c>
       <c r="K11">
-        <v>4202.0</v>
+        <v>4202</v>
       </c>
       <c r="L11">
-        <v>2489.0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" dyDescent="0.2">
+        <v>2489</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>2</v>
       </c>
       <c r="B12" s="8">
         <v>4</v>
       </c>
-      <c r="C12" t="s" s="2">
+      <c r="C12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D12" t="s" s="1">
+      <c r="D12" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E12">
-        <v>103.0</v>
+        <v>103</v>
       </c>
       <c r="F12">
-        <v>110.0</v>
+        <v>110</v>
       </c>
       <c r="G12">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="H12">
         <v>4.7</v>
       </c>
       <c r="I12">
-        <v>2090.0</v>
+        <v>2090</v>
       </c>
       <c r="J12">
-        <v>945.0</v>
+        <v>945</v>
       </c>
       <c r="K12">
-        <v>3035.0</v>
+        <v>3035</v>
       </c>
       <c r="L12">
-        <v>2090.0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" dyDescent="0.2">
+        <v>2090</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>2</v>
       </c>
       <c r="B13" s="8">
         <v>5</v>
       </c>
-      <c r="C13" t="s" s="2">
+      <c r="C13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D13" t="s" s="1">
+      <c r="D13" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E13">
-        <v>89.0</v>
+        <v>89</v>
       </c>
       <c r="F13">
-        <v>80.0</v>
+        <v>80</v>
       </c>
       <c r="G13">
-        <v>16.0</v>
+        <v>16</v>
       </c>
       <c r="H13">
         <v>5.6</v>
       </c>
       <c r="I13">
-        <v>1520.0</v>
+        <v>1520</v>
       </c>
       <c r="J13">
-        <v>852.0</v>
+        <v>852</v>
       </c>
       <c r="K13">
-        <v>2372.0</v>
+        <v>2372</v>
       </c>
       <c r="L13">
-        <v>1520.0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" dyDescent="0.2">
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>2</v>
       </c>
       <c r="B14" s="8">
         <v>6</v>
       </c>
-      <c r="C14" t="s" s="2">
+      <c r="C14" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D14" t="s" s="1">
+      <c r="D14" s="1" t="s">
         <v>56</v>
       </c>
       <c r="E14">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="F14">
-        <v>98.0</v>
+        <v>98</v>
       </c>
       <c r="G14">
-        <v>19.6</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="H14">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I14">
-        <v>1862.0</v>
+        <v>1862</v>
       </c>
       <c r="J14">
-        <v>938.0</v>
+        <v>938</v>
       </c>
       <c r="K14">
-        <v>2800.0</v>
+        <v>2800</v>
       </c>
       <c r="L14">
-        <v>1862.0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" dyDescent="0.2">
+        <v>1862</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>2</v>
       </c>
       <c r="B15" s="8">
         <v>7</v>
       </c>
-      <c r="C15" t="s" s="2">
+      <c r="C15" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D15" t="s" s="11">
+      <c r="D15" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E15">
-        <v>138.0</v>
+        <v>138</v>
       </c>
       <c r="F15">
-        <v>151.0</v>
+        <v>151</v>
       </c>
       <c r="G15">
         <v>30.2</v>
       </c>
       <c r="H15">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I15">
-        <v>2869.0</v>
+        <v>2869</v>
       </c>
       <c r="J15">
-        <v>1258.0</v>
+        <v>1258</v>
       </c>
       <c r="K15">
-        <v>4127.0</v>
+        <v>4127</v>
       </c>
       <c r="L15">
-        <v>2869.0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" dyDescent="0.2">
+        <v>2869</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>2</v>
       </c>
       <c r="B16" s="8">
         <v>8</v>
       </c>
-      <c r="C16" t="s" s="2">
+      <c r="C16" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D16" t="s" s="1">
+      <c r="D16" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E16">
-        <v>55.0</v>
+        <v>55</v>
       </c>
       <c r="F16">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="G16">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="H16">
         <v>6.9</v>
       </c>
       <c r="I16">
-        <v>760.0</v>
+        <v>760</v>
       </c>
       <c r="J16">
-        <v>548.0</v>
+        <v>548</v>
       </c>
       <c r="K16">
-        <v>1308.0</v>
+        <v>1308</v>
       </c>
       <c r="L16">
-        <v>760.0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" dyDescent="0.2">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>2</v>
       </c>
       <c r="B17" s="8">
         <v>9</v>
       </c>
-      <c r="C17" t="s" s="2">
+      <c r="C17" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D17" t="s" s="1">
+      <c r="D17" s="1" t="s">
         <v>59</v>
       </c>
       <c r="E17">
-        <v>38.0</v>
+        <v>38</v>
       </c>
       <c r="F17">
-        <v>26.0</v>
+        <v>26</v>
       </c>
       <c r="G17">
         <v>5.2</v>
@@ -1549,150 +1548,150 @@
         <v>7.3</v>
       </c>
       <c r="I17">
-        <v>494.0</v>
+        <v>494</v>
       </c>
       <c r="J17">
-        <v>383.0</v>
+        <v>383</v>
       </c>
       <c r="K17">
-        <v>877.0</v>
+        <v>877</v>
       </c>
       <c r="L17">
-        <v>494.0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" dyDescent="0.2">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>2</v>
       </c>
       <c r="B18" s="8">
         <v>10</v>
       </c>
-      <c r="C18" t="s" s="2">
+      <c r="C18" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D18" t="s" s="1">
+      <c r="D18" s="1" t="s">
         <v>60</v>
       </c>
       <c r="E18">
-        <v>205.0</v>
+        <v>205</v>
       </c>
       <c r="F18">
-        <v>196.0</v>
+        <v>196</v>
       </c>
       <c r="G18">
-        <v>39.2</v>
+        <v>39.200000000000003</v>
       </c>
       <c r="H18">
         <v>5.2</v>
       </c>
       <c r="I18">
-        <v>3724.0</v>
+        <v>3724</v>
       </c>
       <c r="J18">
-        <v>1934.0</v>
+        <v>1934</v>
       </c>
       <c r="K18">
-        <v>5658.0</v>
+        <v>5658</v>
       </c>
       <c r="L18">
-        <v>3724.0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" dyDescent="0.2">
+        <v>3724</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>3</v>
       </c>
       <c r="B19" s="8">
         <v>4</v>
       </c>
-      <c r="C19" t="s" s="2">
+      <c r="C19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D19" t="s" s="1">
+      <c r="D19" s="1" t="s">
         <v>54</v>
       </c>
       <c r="E19">
-        <v>215.0</v>
+        <v>215</v>
       </c>
       <c r="F19">
-        <v>77.0</v>
+        <v>77</v>
       </c>
       <c r="G19">
         <v>15.4</v>
       </c>
       <c r="H19">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="I19">
-        <v>1463.0</v>
+        <v>1463</v>
       </c>
       <c r="J19">
-        <v>2329.0</v>
+        <v>2329</v>
       </c>
       <c r="K19">
-        <v>3792.0</v>
+        <v>3792</v>
       </c>
       <c r="L19">
-        <v>2329.0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" dyDescent="0.2">
+        <v>2329</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>3</v>
       </c>
       <c r="B20" s="8">
         <v>5</v>
       </c>
-      <c r="C20" t="s" s="2">
+      <c r="C20" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D20" t="s" s="1">
+      <c r="D20" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E20">
-        <v>113.0</v>
+        <v>113</v>
       </c>
       <c r="F20">
-        <v>63.0</v>
+        <v>63</v>
       </c>
       <c r="G20">
         <v>12.6</v>
       </c>
       <c r="H20">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="I20">
-        <v>1197.0</v>
+        <v>1197</v>
       </c>
       <c r="J20">
-        <v>1171.0</v>
+        <v>1171</v>
       </c>
       <c r="K20">
-        <v>2368.0</v>
+        <v>2368</v>
       </c>
       <c r="L20">
-        <v>1197.0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" dyDescent="0.2">
+        <v>1197</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>3</v>
       </c>
       <c r="B21" s="8">
         <v>6</v>
       </c>
-      <c r="C21" t="s" s="2">
+      <c r="C21" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D21" t="s" s="1">
+      <c r="D21" s="1" t="s">
         <v>56</v>
       </c>
       <c r="E21">
-        <v>192.0</v>
+        <v>192</v>
       </c>
       <c r="F21">
-        <v>126.0</v>
+        <v>126</v>
       </c>
       <c r="G21">
         <v>25.2</v>
@@ -1701,36 +1700,36 @@
         <v>7.6</v>
       </c>
       <c r="I21">
-        <v>2394.0</v>
+        <v>2394</v>
       </c>
       <c r="J21">
-        <v>1946.0</v>
+        <v>1946</v>
       </c>
       <c r="K21">
-        <v>4340.0</v>
+        <v>4340</v>
       </c>
       <c r="L21">
-        <v>2394.0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" dyDescent="0.2">
+        <v>2394</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A22">
         <v>3</v>
       </c>
       <c r="B22" s="8">
         <v>7</v>
       </c>
-      <c r="C22" t="s" s="2">
+      <c r="C22" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D22" t="s" s="11">
+      <c r="D22" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E22">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="F22">
-        <v>167.0</v>
+        <v>167</v>
       </c>
       <c r="G22">
         <v>33.4</v>
@@ -1739,112 +1738,112 @@
         <v>7.5</v>
       </c>
       <c r="I22">
-        <v>3173.0</v>
+        <v>3173</v>
       </c>
       <c r="J22">
-        <v>2527.0</v>
+        <v>2527</v>
       </c>
       <c r="K22">
-        <v>5700.0</v>
+        <v>5700</v>
       </c>
       <c r="L22">
-        <v>3173.0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" dyDescent="0.2">
+        <v>3173</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>3</v>
       </c>
       <c r="B23" s="8">
         <v>8</v>
       </c>
-      <c r="C23" t="s" s="2">
+      <c r="C23" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D23" t="s" s="1">
+      <c r="D23" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E23">
-        <v>130.0</v>
+        <v>130</v>
       </c>
       <c r="F23">
-        <v>97.0</v>
+        <v>97</v>
       </c>
       <c r="G23">
-        <v>19.4</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="H23">
         <v>6.7</v>
       </c>
       <c r="I23">
-        <v>1843.0</v>
+        <v>1843</v>
       </c>
       <c r="J23">
-        <v>1290.0</v>
+        <v>1290</v>
       </c>
       <c r="K23">
-        <v>3133.0</v>
+        <v>3133</v>
       </c>
       <c r="L23">
-        <v>1843.0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" dyDescent="0.2">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>3</v>
       </c>
       <c r="B24" s="8">
         <v>9</v>
       </c>
-      <c r="C24" t="s" s="2">
+      <c r="C24" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D24" t="s" s="1">
+      <c r="D24" s="1" t="s">
         <v>59</v>
       </c>
       <c r="E24">
-        <v>142.0</v>
+        <v>142</v>
       </c>
       <c r="F24">
-        <v>105.0</v>
+        <v>105</v>
       </c>
       <c r="G24">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="H24">
         <v>6.8</v>
       </c>
       <c r="I24">
-        <v>1995.0</v>
+        <v>1995</v>
       </c>
       <c r="J24">
-        <v>1412.0</v>
+        <v>1412</v>
       </c>
       <c r="K24">
-        <v>3407.0</v>
+        <v>3407</v>
       </c>
       <c r="L24">
-        <v>1995.0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" dyDescent="0.2">
+        <v>1995</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>3</v>
       </c>
       <c r="B25" s="8">
         <v>10</v>
       </c>
-      <c r="C25" t="s" s="2">
+      <c r="C25" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D25" t="s" s="1">
+      <c r="D25" s="1" t="s">
         <v>60</v>
       </c>
       <c r="E25">
-        <v>89.0</v>
+        <v>89</v>
       </c>
       <c r="F25">
-        <v>68.0</v>
+        <v>68</v>
       </c>
       <c r="G25">
         <v>13.6</v>
@@ -1853,188 +1852,188 @@
         <v>6.5</v>
       </c>
       <c r="I25">
-        <v>1292.0</v>
+        <v>1292</v>
       </c>
       <c r="J25">
-        <v>880.0</v>
+        <v>880</v>
       </c>
       <c r="K25">
-        <v>2172.0</v>
+        <v>2172</v>
       </c>
       <c r="L25">
-        <v>1292.0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" dyDescent="0.2">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A26">
         <v>4</v>
       </c>
       <c r="B26" s="8">
         <v>5</v>
       </c>
-      <c r="C26" t="s" s="1">
+      <c r="C26" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D26" t="s" s="1">
+      <c r="D26" s="1" t="s">
         <v>55</v>
       </c>
       <c r="E26">
-        <v>130.0</v>
+        <v>130</v>
       </c>
       <c r="F26">
-        <v>93.0</v>
+        <v>93</v>
       </c>
       <c r="G26">
-        <v>18.6</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="H26">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="I26">
-        <v>1767.0</v>
+        <v>1767</v>
       </c>
       <c r="J26">
-        <v>1300.0</v>
+        <v>1300</v>
       </c>
       <c r="K26">
-        <v>3067.0</v>
+        <v>3067</v>
       </c>
       <c r="L26">
-        <v>1767.0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" dyDescent="0.2">
+        <v>1767</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>4</v>
       </c>
       <c r="B27" s="8">
         <v>6</v>
       </c>
-      <c r="C27" t="s" s="1">
+      <c r="C27" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D27" t="s" s="1">
+      <c r="D27" s="1" t="s">
         <v>56</v>
       </c>
       <c r="E27">
-        <v>149.0</v>
+        <v>149</v>
       </c>
       <c r="F27">
-        <v>161.0</v>
+        <v>161</v>
       </c>
       <c r="G27">
-        <v>32.2</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="H27">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I27">
-        <v>3059.0</v>
+        <v>3059</v>
       </c>
       <c r="J27">
-        <v>1363.0</v>
+        <v>1363</v>
       </c>
       <c r="K27">
-        <v>4422.0</v>
+        <v>4422</v>
       </c>
       <c r="L27">
-        <v>3059.0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" dyDescent="0.2">
+        <v>3059</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>4</v>
       </c>
       <c r="B28" s="8">
         <v>7</v>
       </c>
-      <c r="C28" t="s" s="1">
+      <c r="C28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D28" t="s" s="11">
+      <c r="D28" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E28">
-        <v>93.0</v>
+        <v>93</v>
       </c>
       <c r="F28">
-        <v>90.0</v>
+        <v>90</v>
       </c>
       <c r="G28">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="H28">
         <v>5.2</v>
       </c>
       <c r="I28">
-        <v>1710.0</v>
+        <v>1710</v>
       </c>
       <c r="J28">
-        <v>875.0</v>
+        <v>875</v>
       </c>
       <c r="K28">
-        <v>2585.0</v>
+        <v>2585</v>
       </c>
       <c r="L28">
-        <v>1710.0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" dyDescent="0.2">
+        <v>1710</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>4</v>
       </c>
       <c r="B29" s="8">
         <v>8</v>
       </c>
-      <c r="C29" t="s" s="1">
+      <c r="C29" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D29" t="s" s="1">
+      <c r="D29" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E29">
-        <v>97.0</v>
+        <v>97</v>
       </c>
       <c r="F29">
-        <v>97.0</v>
+        <v>97</v>
       </c>
       <c r="G29">
-        <v>19.4</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="H29">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="I29">
-        <v>1843.0</v>
+        <v>1843</v>
       </c>
       <c r="J29">
-        <v>905.0</v>
+        <v>905</v>
       </c>
       <c r="K29">
-        <v>2748.0</v>
+        <v>2748</v>
       </c>
       <c r="L29">
-        <v>1843.0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" dyDescent="0.2">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>4</v>
       </c>
       <c r="B30" s="8">
         <v>9</v>
       </c>
-      <c r="C30" t="s" s="1">
+      <c r="C30" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D30" t="s" s="1">
+      <c r="D30" s="1" t="s">
         <v>59</v>
       </c>
       <c r="E30">
-        <v>76.0</v>
+        <v>76</v>
       </c>
       <c r="F30">
-        <v>91.0</v>
+        <v>91</v>
       </c>
       <c r="G30">
         <v>18.2</v>
@@ -2043,226 +2042,226 @@
         <v>4.2</v>
       </c>
       <c r="I30">
-        <v>1729.0</v>
+        <v>1729</v>
       </c>
       <c r="J30">
-        <v>674.0</v>
+        <v>674</v>
       </c>
       <c r="K30">
-        <v>2403.0</v>
+        <v>2403</v>
       </c>
       <c r="L30">
-        <v>1729.0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" dyDescent="0.2">
+        <v>1729</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A31">
         <v>4</v>
       </c>
       <c r="B31" s="8">
         <v>10</v>
       </c>
-      <c r="C31" t="s" s="1">
+      <c r="C31" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D31" t="s" s="1">
+      <c r="D31" s="1" t="s">
         <v>60</v>
       </c>
       <c r="E31">
-        <v>246.0</v>
+        <v>246</v>
       </c>
       <c r="F31">
-        <v>110.0</v>
+        <v>110</v>
       </c>
       <c r="G31">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="H31">
         <v>11.2</v>
       </c>
       <c r="I31">
-        <v>2090.0</v>
+        <v>2090</v>
       </c>
       <c r="J31">
-        <v>2613.0</v>
+        <v>2613</v>
       </c>
       <c r="K31">
-        <v>4703.0</v>
+        <v>4703</v>
       </c>
       <c r="L31">
-        <v>2613.0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" dyDescent="0.2">
+        <v>2613</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A32">
         <v>5</v>
       </c>
       <c r="B32" s="8">
         <v>6</v>
       </c>
-      <c r="C32" t="s" s="1">
+      <c r="C32" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D32" t="s" s="1">
+      <c r="D32" s="1" t="s">
         <v>56</v>
       </c>
       <c r="E32">
-        <v>110.0</v>
+        <v>110</v>
       </c>
       <c r="F32">
-        <v>70.0</v>
+        <v>70</v>
       </c>
       <c r="G32">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="H32">
         <v>7.9</v>
       </c>
       <c r="I32">
-        <v>1330.0</v>
+        <v>1330</v>
       </c>
       <c r="J32">
-        <v>1120.0</v>
+        <v>1120</v>
       </c>
       <c r="K32">
-        <v>2450.0</v>
+        <v>2450</v>
       </c>
       <c r="L32">
-        <v>1330.0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" dyDescent="0.2">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A33" s="10">
         <v>5</v>
       </c>
       <c r="B33" s="8">
         <v>7</v>
       </c>
-      <c r="C33" t="s" s="1">
+      <c r="C33" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D33" t="s" s="11">
+      <c r="D33" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E33">
-        <v>168.0</v>
+        <v>168</v>
       </c>
       <c r="F33">
-        <v>173.0</v>
+        <v>173</v>
       </c>
       <c r="G33">
         <v>34.6</v>
       </c>
       <c r="H33">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I33">
-        <v>3287.0</v>
+        <v>3287</v>
       </c>
       <c r="J33">
-        <v>1556.0</v>
+        <v>1556</v>
       </c>
       <c r="K33">
-        <v>4843.0</v>
+        <v>4843</v>
       </c>
       <c r="L33">
-        <v>3287.0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" dyDescent="0.2">
+        <v>3287</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A34">
         <v>5</v>
       </c>
       <c r="B34" s="8">
         <v>8</v>
       </c>
-      <c r="C34" t="s" s="1">
+      <c r="C34" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D34" t="s" s="1">
+      <c r="D34" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E34">
-        <v>48.0</v>
+        <v>48</v>
       </c>
       <c r="F34">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="G34">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="H34">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="I34">
-        <v>760.0</v>
+        <v>760</v>
       </c>
       <c r="J34">
-        <v>467.0</v>
+        <v>467</v>
       </c>
       <c r="K34">
-        <v>1227.0</v>
+        <v>1227</v>
       </c>
       <c r="L34">
-        <v>760.0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" dyDescent="0.2">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A35">
         <v>5</v>
       </c>
       <c r="B35" s="8">
         <v>9</v>
       </c>
-      <c r="C35" t="s" s="1">
+      <c r="C35" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D35" t="s" s="1">
+      <c r="D35" s="1" t="s">
         <v>59</v>
       </c>
       <c r="E35">
-        <v>60.0</v>
+        <v>60</v>
       </c>
       <c r="F35">
-        <v>55.0</v>
+        <v>55</v>
       </c>
       <c r="G35">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="H35">
         <v>5.5</v>
       </c>
       <c r="I35">
-        <v>1045.0</v>
+        <v>1045</v>
       </c>
       <c r="J35">
-        <v>572.0</v>
+        <v>572</v>
       </c>
       <c r="K35">
-        <v>1617.0</v>
+        <v>1617</v>
       </c>
       <c r="L35">
-        <v>1045.0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" dyDescent="0.2">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>5</v>
       </c>
       <c r="B36" s="8">
         <v>10</v>
       </c>
-      <c r="C36" t="s" s="1">
+      <c r="C36" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D36" t="s" s="1">
+      <c r="D36" s="1" t="s">
         <v>60</v>
       </c>
       <c r="E36">
-        <v>145.0</v>
+        <v>145</v>
       </c>
       <c r="F36">
-        <v>131.0</v>
+        <v>131</v>
       </c>
       <c r="G36">
         <v>26.2</v>
@@ -2271,74 +2270,74 @@
         <v>5.5</v>
       </c>
       <c r="I36">
-        <v>2489.0</v>
+        <v>2489</v>
       </c>
       <c r="J36">
-        <v>1386.0</v>
+        <v>1386</v>
       </c>
       <c r="K36">
-        <v>3875.0</v>
+        <v>3875</v>
       </c>
       <c r="L36">
-        <v>2489.0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" dyDescent="0.2">
+        <v>2489</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A37">
         <v>6</v>
       </c>
       <c r="B37" s="8">
         <v>7</v>
       </c>
-      <c r="C37" t="s" s="1">
+      <c r="C37" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D37" t="s" s="11">
+      <c r="D37" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E37">
-        <v>185.0</v>
+        <v>185</v>
       </c>
       <c r="F37">
-        <v>232.0</v>
+        <v>232</v>
       </c>
       <c r="G37">
         <v>46.4</v>
       </c>
       <c r="H37">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I37">
-        <v>4408.0</v>
+        <v>4408</v>
       </c>
       <c r="J37">
-        <v>1617.0</v>
+        <v>1617</v>
       </c>
       <c r="K37">
-        <v>6025.0</v>
+        <v>6025</v>
       </c>
       <c r="L37">
-        <v>4408.0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" dyDescent="0.2">
+        <v>4408</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A38">
         <v>6</v>
       </c>
       <c r="B38" s="8">
         <v>8</v>
       </c>
-      <c r="C38" t="s" s="1">
+      <c r="C38" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D38" t="s" s="1">
+      <c r="D38" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E38">
-        <v>77.0</v>
+        <v>77</v>
       </c>
       <c r="F38">
-        <v>72.0</v>
+        <v>72</v>
       </c>
       <c r="G38">
         <v>14.4</v>
@@ -2347,74 +2346,74 @@
         <v>5.3</v>
       </c>
       <c r="I38">
-        <v>1368.0</v>
+        <v>1368</v>
       </c>
       <c r="J38">
-        <v>730.0</v>
+        <v>730</v>
       </c>
       <c r="K38">
-        <v>2098.0</v>
+        <v>2098</v>
       </c>
       <c r="L38">
-        <v>1368.0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" dyDescent="0.2">
+        <v>1368</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>6</v>
       </c>
       <c r="B39" s="8">
         <v>9</v>
       </c>
-      <c r="C39" t="s" s="1">
+      <c r="C39" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D39" t="s" s="1">
+      <c r="D39" s="1" t="s">
         <v>59</v>
       </c>
       <c r="E39">
-        <v>78.0</v>
+        <v>78</v>
       </c>
       <c r="F39">
-        <v>89.0</v>
+        <v>89</v>
       </c>
       <c r="G39">
         <v>17.8</v>
       </c>
       <c r="H39">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="I39">
-        <v>1691.0</v>
+        <v>1691</v>
       </c>
       <c r="J39">
-        <v>702.0</v>
+        <v>702</v>
       </c>
       <c r="K39">
-        <v>2393.0</v>
+        <v>2393</v>
       </c>
       <c r="L39">
-        <v>1691.0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" dyDescent="0.2">
+        <v>1691</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A40">
         <v>6</v>
       </c>
       <c r="B40" s="8">
         <v>10</v>
       </c>
-      <c r="C40" t="s" s="1">
+      <c r="C40" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D40" t="s" s="1">
+      <c r="D40" s="1" t="s">
         <v>60</v>
       </c>
       <c r="E40">
-        <v>224.0</v>
+        <v>224</v>
       </c>
       <c r="F40">
-        <v>192.0</v>
+        <v>192</v>
       </c>
       <c r="G40">
         <v>38.4</v>
@@ -2423,74 +2422,74 @@
         <v>5.8</v>
       </c>
       <c r="I40">
-        <v>3648.0</v>
+        <v>3648</v>
       </c>
       <c r="J40">
-        <v>2165.0</v>
+        <v>2165</v>
       </c>
       <c r="K40">
-        <v>5813.0</v>
+        <v>5813</v>
       </c>
       <c r="L40">
-        <v>3648.0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" dyDescent="0.2">
+        <v>3648</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>7</v>
       </c>
       <c r="B41" s="8">
         <v>8</v>
       </c>
-      <c r="C41" t="s" s="1">
+      <c r="C41" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D41" t="s" s="1">
+      <c r="D41" s="1" t="s">
         <v>58</v>
       </c>
       <c r="E41">
-        <v>131.0</v>
+        <v>131</v>
       </c>
       <c r="F41">
-        <v>160.0</v>
+        <v>160</v>
       </c>
       <c r="G41">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="H41">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I41">
-        <v>3040.0</v>
+        <v>3040</v>
       </c>
       <c r="J41">
-        <v>1155.0</v>
+        <v>1155</v>
       </c>
       <c r="K41">
-        <v>4195.0</v>
+        <v>4195</v>
       </c>
       <c r="L41">
-        <v>3040.0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" dyDescent="0.2">
+        <v>3040</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>7</v>
       </c>
       <c r="B42" s="8">
         <v>9</v>
       </c>
-      <c r="C42" t="s" s="1">
+      <c r="C42" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D42" t="s" s="1">
+      <c r="D42" s="1" t="s">
         <v>59</v>
       </c>
       <c r="E42">
-        <v>110.0</v>
+        <v>110</v>
       </c>
       <c r="F42">
-        <v>146.0</v>
+        <v>146</v>
       </c>
       <c r="G42">
         <v>29.2</v>
@@ -2499,36 +2498,36 @@
         <v>3.8</v>
       </c>
       <c r="I42">
-        <v>2774.0</v>
+        <v>2774</v>
       </c>
       <c r="J42">
-        <v>943.0</v>
+        <v>943</v>
       </c>
       <c r="K42">
-        <v>3717.0</v>
+        <v>3717</v>
       </c>
       <c r="L42">
-        <v>2774.0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" dyDescent="0.2">
+        <v>2774</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A43">
         <v>7</v>
       </c>
       <c r="B43" s="8">
         <v>10</v>
       </c>
-      <c r="C43" t="s" s="1">
+      <c r="C43" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D43" t="s" s="1">
+      <c r="D43" s="1" t="s">
         <v>60</v>
       </c>
       <c r="E43">
-        <v>280.0</v>
+        <v>280</v>
       </c>
       <c r="F43">
-        <v>187.0</v>
+        <v>187</v>
       </c>
       <c r="G43">
         <v>37.4</v>
@@ -2537,36 +2536,36 @@
         <v>7.5</v>
       </c>
       <c r="I43">
-        <v>3553.0</v>
+        <v>3553</v>
       </c>
       <c r="J43">
-        <v>2830.0</v>
+        <v>2830</v>
       </c>
       <c r="K43">
-        <v>6383.0</v>
+        <v>6383</v>
       </c>
       <c r="L43">
-        <v>3553.0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" dyDescent="0.2">
+        <v>3553</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A44">
         <v>8</v>
       </c>
       <c r="B44" s="8">
         <v>9</v>
       </c>
-      <c r="C44" t="s" s="1">
+      <c r="C44" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D44" t="s" s="1">
+      <c r="D44" s="1" t="s">
         <v>59</v>
       </c>
       <c r="E44">
-        <v>26.0</v>
+        <v>26</v>
       </c>
       <c r="F44">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="G44">
         <v>3.8</v>
@@ -2575,95 +2574,95 @@
         <v>6.8</v>
       </c>
       <c r="I44">
-        <v>361.0</v>
+        <v>361</v>
       </c>
       <c r="J44">
-        <v>259.0</v>
+        <v>259</v>
       </c>
       <c r="K44">
-        <v>620.0</v>
+        <v>620</v>
       </c>
       <c r="L44">
-        <v>361.0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" dyDescent="0.2">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A45">
         <v>8</v>
       </c>
       <c r="B45" s="8">
         <v>10</v>
       </c>
-      <c r="C45" t="s" s="1">
+      <c r="C45" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D45" t="s" s="1">
+      <c r="D45" s="1" t="s">
         <v>60</v>
       </c>
       <c r="E45">
-        <v>163.0</v>
+        <v>163</v>
       </c>
       <c r="F45">
-        <v>164.0</v>
+        <v>164</v>
       </c>
       <c r="G45">
-        <v>32.8</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="H45">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="I45">
-        <v>3116.0</v>
+        <v>3116</v>
       </c>
       <c r="J45">
-        <v>1519.0</v>
+        <v>1519</v>
       </c>
       <c r="K45">
-        <v>4635.0</v>
+        <v>4635</v>
       </c>
       <c r="L45">
-        <v>3116.0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" dyDescent="0.2">
+        <v>3116</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A46">
         <v>9</v>
       </c>
       <c r="B46" s="8">
         <v>10</v>
       </c>
-      <c r="C46" t="s" s="1">
+      <c r="C46" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D46" t="s" s="1">
+      <c r="D46" s="1" t="s">
         <v>60</v>
       </c>
       <c r="E46">
-        <v>175.0</v>
+        <v>175</v>
       </c>
       <c r="F46">
-        <v>170.0</v>
+        <v>170</v>
       </c>
       <c r="G46">
-        <v>34.0</v>
+        <v>34</v>
       </c>
       <c r="H46">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I46">
-        <v>3230.0</v>
+        <v>3230</v>
       </c>
       <c r="J46">
-        <v>1645.0</v>
+        <v>1645</v>
       </c>
       <c r="K46">
-        <v>4875.0</v>
+        <v>4875</v>
       </c>
       <c r="L46">
-        <v>3230.0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" dyDescent="0.2">
+        <v>3230</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A47">
         <v>1</v>
       </c>
@@ -2697,7 +2696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:16" dyDescent="0.2">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A48">
         <v>2</v>
       </c>
@@ -2731,7 +2730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:16" dyDescent="0.2">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A49">
         <v>3</v>
       </c>
@@ -2765,7 +2764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:16" dyDescent="0.2">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A50">
         <v>4</v>
       </c>
@@ -2799,7 +2798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:16" dyDescent="0.2">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A51">
         <v>5</v>
       </c>
@@ -2833,7 +2832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:16" dyDescent="0.2">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A52">
         <v>6</v>
       </c>
@@ -2865,7 +2864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:16" dyDescent="0.2">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A53">
         <v>7</v>
       </c>
@@ -2897,7 +2896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:16" dyDescent="0.2">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A54">
         <v>8</v>
       </c>
@@ -2929,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:16" dyDescent="0.2">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A55">
         <v>9</v>
       </c>
@@ -2961,7 +2960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:16" dyDescent="0.2">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A56">
         <v>10</v>
       </c>
@@ -2993,13 +2992,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:16" dyDescent="0.2">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.4">
       <c r="G57" s="2"/>
     </row>
-    <row r="58" spans="1:16" dyDescent="0.2">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.4">
       <c r="G58" s="1"/>
     </row>
-    <row r="59" spans="1:16" dyDescent="0.2">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.4">
       <c r="G59" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Excel file references and adjust parameters for data loading
</commit_message>
<xml_diff>
--- a/inputData/Parameters.xlsx
+++ b/inputData/Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/inputData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F278866-8B49-0647-A835-544B4947017F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6178247B-1275-40E8-B67D-0E5573380FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16320" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="9" r:id="rId1"/>
@@ -647,18 +647,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15C49E0-A7B4-734A-8962-DC2A879F4079}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.6640625" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -669,7 +669,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -680,7 +680,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -691,7 +691,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -702,7 +702,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -713,7 +713,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -724,7 +724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -736,7 +736,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -747,7 +747,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -758,7 +758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>45</v>
       </c>
@@ -769,7 +769,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -780,7 +780,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -791,7 +791,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -803,7 +803,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -815,7 +815,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -827,18 +827,18 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>6</v>
       </c>
       <c r="B17" s="4">
-        <v>780</v>
+        <v>120</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -858,7 +858,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF0D5EA-53B5-1240-9D84-6FE223856A18}">
   <dimension ref="A1:P59"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="17.1640625" customWidth="1"/>
@@ -868,7 +868,7 @@
     <col min="8" max="8" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A1" s="9" t="s">
         <v>36</v>
       </c>
@@ -913,7 +913,7 @@
       </c>
       <c r="P1" s="6"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -960,7 +960,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1099,7 +1099,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>1</v>
       </c>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="O6" s="4"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="O7" s="4"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>1</v>
       </c>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="O8" s="4"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>1</v>
       </c>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="O9" s="4"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>1</v>
       </c>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="O10" s="4"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>2489</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>2</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>2090</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>1862</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>2869</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>2</v>
       </c>
@@ -1598,7 +1598,7 @@
         <v>3724</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>3</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>2329</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>3</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>2394</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A22">
         <v>3</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>3173</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>3</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>1843</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>3</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>3</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>1292</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A26">
         <v>4</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>1767</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>4</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>3059</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>4</v>
       </c>
@@ -1978,7 +1978,7 @@
         <v>1710</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>4</v>
       </c>
@@ -2016,7 +2016,7 @@
         <v>1843</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>4</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>1729</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A31">
         <v>4</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>2613</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A32">
         <v>5</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A33" s="10">
         <v>5</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>3287</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A34">
         <v>5</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A35">
         <v>5</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>5</v>
       </c>
@@ -2282,7 +2282,7 @@
         <v>2489</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A37">
         <v>6</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>4408</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A38">
         <v>6</v>
       </c>
@@ -2358,7 +2358,7 @@
         <v>1368</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>6</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>1691</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A40">
         <v>6</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>3648</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>7</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>3040</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>7</v>
       </c>
@@ -2510,7 +2510,7 @@
         <v>2774</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A43">
         <v>7</v>
       </c>
@@ -2548,7 +2548,7 @@
         <v>3553</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A44">
         <v>8</v>
       </c>
@@ -2586,7 +2586,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A45">
         <v>8</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>3116</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A46">
         <v>9</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>3230</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A47">
         <v>1</v>
       </c>
@@ -2696,7 +2696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A48">
         <v>2</v>
       </c>
@@ -2730,7 +2730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A49">
         <v>3</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A50">
         <v>4</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A51">
         <v>5</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A52">
         <v>6</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A53">
         <v>7</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A54">
         <v>8</v>
       </c>
@@ -2928,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A55">
         <v>9</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A56">
         <v>10</v>
       </c>
@@ -2992,13 +2992,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.4">
       <c r="G57" s="2"/>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.4">
       <c r="G58" s="1"/>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.4">
       <c r="G59" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data loading functions to use new Excel file structure
</commit_message>
<xml_diff>
--- a/inputData/Parameters.xlsx
+++ b/inputData/Parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6178247B-1275-40E8-B67D-0E5573380FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{600B90F6-DDA5-479D-AA66-1FABE0EB37D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
@@ -707,7 +707,7 @@
         <v>17</v>
       </c>
       <c r="B6" s="4">
-        <v>1.51</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Added KPI functions and a script to run multiple deterministic runs
</commit_message>
<xml_diff>
--- a/inputData/Parameters.xlsx
+++ b/inputData/Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/inputData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE494151-0397-8E43-9CE6-8F1B08E35F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14C88F75-73F9-431A-9C84-FF9086595067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2000" yWindow="500" windowWidth="19420" windowHeight="16320" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="9" r:id="rId1"/>
@@ -647,18 +647,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15C49E0-A7B4-734A-8962-DC2A879F4079}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" style="4"/>
+    <col min="1" max="1" width="22.625" customWidth="1"/>
+    <col min="2" max="2" width="10.875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -669,7 +669,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -680,7 +680,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -691,7 +691,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -702,7 +702,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -713,7 +713,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -724,7 +724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -736,7 +736,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -747,7 +747,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -758,7 +758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -769,7 +769,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -780,7 +780,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -791,7 +791,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -803,7 +803,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -815,7 +815,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -827,18 +827,18 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>6</v>
       </c>
       <c r="B17" s="4">
-        <v>120</v>
+        <v>780</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -858,17 +858,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF0D5EA-53B5-1240-9D84-6FE223856A18}">
   <dimension ref="A1:P59"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="17.1640625" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="17.125" customWidth="1"/>
+    <col min="5" max="5" width="12.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>36</v>
       </c>
@@ -913,7 +913,7 @@
       </c>
       <c r="P1" s="6"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -960,7 +960,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1099,7 +1099,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="O6" s="4"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="O7" s="4"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="O8" s="4"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="O9" s="4"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="O10" s="4"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>2489</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>2090</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>1862</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>2869</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2</v>
       </c>
@@ -1598,7 +1598,7 @@
         <v>3724</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>2329</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>3</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>2394</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>3</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>3173</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>3</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>1843</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>3</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>3</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>1292</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>4</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>1767</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>4</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>3059</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>4</v>
       </c>
@@ -1978,7 +1978,7 @@
         <v>1710</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>4</v>
       </c>
@@ -2016,7 +2016,7 @@
         <v>1843</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>4</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>1729</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>4</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>2613</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>5</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="10">
         <v>5</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>3287</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>5</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>5</v>
       </c>
@@ -2244,7 +2244,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>5</v>
       </c>
@@ -2282,7 +2282,7 @@
         <v>2489</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>6</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>4408</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>6</v>
       </c>
@@ -2358,7 +2358,7 @@
         <v>1368</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>6</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>1691</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>6</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>3648</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>7</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>3040</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>7</v>
       </c>
@@ -2510,7 +2510,7 @@
         <v>2774</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>7</v>
       </c>
@@ -2548,7 +2548,7 @@
         <v>3553</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>8</v>
       </c>
@@ -2586,7 +2586,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>8</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>3116</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>9</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>3230</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>1</v>
       </c>
@@ -2696,7 +2696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2</v>
       </c>
@@ -2730,7 +2730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>3</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>4</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>5</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>6</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>7</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>8</v>
       </c>
@@ -2928,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>9</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>10</v>
       </c>
@@ -2992,13 +2992,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G57" s="2"/>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G58" s="1"/>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G59" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Zero cost for i to i VP
</commit_message>
<xml_diff>
--- a/inputData/Parameters.xlsx
+++ b/inputData/Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/inputData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0218802E-FB40-954D-9A70-48D7F6E8A911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B1B232-F1DE-494C-9564-42A59FF0DB02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1180" windowWidth="28800" windowHeight="15280" activeTab="1" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="9" r:id="rId1"/>
@@ -509,7 +509,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3CFD079E-5109-8F49-8A19-E09E2BEBBC8C}" name="Table13" displayName="Table13" ref="A1:N56" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6" headerRowCellStyle="Comma" dataCellStyle="Comma">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3CFD079E-5109-8F49-8A19-E09E2BEBBC8C}" name="Table13" displayName="Table13" ref="A1:N56" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
   <autoFilter ref="A1:N56" xr:uid="{CEDCB4F7-0752-8449-BE87-89650C1E9E7C}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{0330B38A-598B-B64A-86F4-FA8E25EAC437}" name="From"/>
@@ -521,15 +521,15 @@
     <tableColumn id="7" xr3:uid="{59F6BECD-EB60-114E-826A-884ADDC4EE72}" name="Km fugleflugt"/>
     <tableColumn id="8" xr3:uid="{605D45AE-CBF2-E342-BA16-1B205DDE6C4E}" name="eVTOL flyvetid (min)"/>
     <tableColumn id="9" xr3:uid="{FCFA00C8-AEDC-F54B-AE4D-2360ACC6025E}" name="Hvor meget hurtigere"/>
-    <tableColumn id="10" xr3:uid="{DBB7D64B-F97D-5C46-B464-1DA11C10DF3A}" name="Pris (Bil udgift)" dataDxfId="4" dataCellStyle="Comma"/>
-    <tableColumn id="11" xr3:uid="{CC283087-BB53-D146-A233-2D178D7E3562}" name="Færge (gns. Gælder kun Bornholm)" dataDxfId="3" dataCellStyle="Comma"/>
-    <tableColumn id="12" xr3:uid="{B4DC4D17-2AE3-D34D-926C-7506AC52E6B8}" name="Base" dataDxfId="2" dataCellStyle="Comma">
+    <tableColumn id="10" xr3:uid="{DBB7D64B-F97D-5C46-B464-1DA11C10DF3A}" name="Pris (Bil udgift)" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{CC283087-BB53-D146-A233-2D178D7E3562}" name="Færge (gns. Gælder kun Bornholm)" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{B4DC4D17-2AE3-D34D-926C-7506AC52E6B8}" name="Base" dataDxfId="2">
       <calculatedColumnFormula>$Q$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{E70B016F-0534-2048-951F-6FD04DC33B7C}" name="Pris (udfra tidsbesparelse)" dataDxfId="1" dataCellStyle="Comma">
+    <tableColumn id="13" xr3:uid="{E70B016F-0534-2048-951F-6FD04DC33B7C}" name="Pris (udfra tidsbesparelse)" dataDxfId="1">
       <calculatedColumnFormula>$Q$4*MAX(F2-G2*$Q$1)*$Q$3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{67EF8C2F-B7CB-8D4A-8447-692E942D0514}" name="fd_sum" dataDxfId="0" dataCellStyle="Comma">
+    <tableColumn id="14" xr3:uid="{67EF8C2F-B7CB-8D4A-8447-692E942D0514}" name="fd_sum" dataDxfId="0">
       <calculatedColumnFormula>SUM(J2:M2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -855,18 +855,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15C49E0-A7B4-734A-8962-DC2A879F4079}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" style="4"/>
+    <col min="1" max="1" width="22.625" customWidth="1"/>
+    <col min="2" max="2" width="10.875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -877,7 +877,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -888,7 +888,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>42</v>
       </c>
@@ -899,7 +899,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -910,7 +910,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -921,7 +921,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -932,7 +932,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -944,7 +944,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -955,7 +955,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -966,7 +966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -977,7 +977,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -988,7 +988,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -999,7 +999,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1023,7 +1023,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -1066,23 +1066,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36FC1A80-FC3B-6349-8B7A-4A1A2A7C8FC7}">
   <dimension ref="A1:R56"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="17.1640625" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="17.125" customWidth="1"/>
+    <col min="5" max="5" width="12.125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5" customWidth="1"/>
-    <col min="7" max="7" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.33203125" customWidth="1"/>
+    <col min="7" max="7" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.375" customWidth="1"/>
     <col min="9" max="9" width="21" style="10" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" style="10" customWidth="1"/>
-    <col min="11" max="11" width="32.1640625" style="10" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" style="10"/>
+    <col min="10" max="10" width="13.625" style="10" customWidth="1"/>
+    <col min="11" max="11" width="32.125" style="10" customWidth="1"/>
+    <col min="12" max="12" width="10.625" style="10"/>
     <col min="13" max="13" width="27" style="10" customWidth="1"/>
-    <col min="14" max="14" width="10.83203125" style="10" customWidth="1"/>
+    <col min="14" max="14" width="10.875" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>33</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1249,7 +1249,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -1420,7 +1420,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>3195.666666666667</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>2678</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>2719.333333333333</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>1020.6666666666667</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>2111.666666666667</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2</v>
       </c>
@@ -1714,7 +1714,7 @@
         <v>1451</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1763,7 +1763,7 @@
         <v>1304.6666666666667</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1861,7 +1861,7 @@
         <v>1833.6666666666665</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1910,7 +1910,7 @@
         <v>4409.3333333333339</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>1245.6666666666667</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>2579</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>3</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>2703.666666666667</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>3</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>1532.3333333333335</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>3</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>2419</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>3</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>3021</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>3</v>
       </c>
@@ -2253,7 +2253,7 @@
         <v>3380.3333333333335</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>3</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>2572.666666666667</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>3</v>
       </c>
@@ -2351,7 +2351,7 @@
         <v>1490.3333333333335</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>4</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>1803.6666666666667</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>4</v>
       </c>
@@ -2449,7 +2449,7 @@
         <v>1977.6666666666665</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>4</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>1378</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>4</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>5017.666666666667</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>4</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>1277</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>4</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>3221</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>5</v>
       </c>
@@ -2694,7 +2694,7 @@
         <v>1632</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
         <v>5</v>
       </c>
@@ -2743,7 +2743,7 @@
         <v>2151.3333333333335</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>5</v>
       </c>
@@ -2792,7 +2792,7 @@
         <v>3846.3333333333335</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>5</v>
       </c>
@@ -2841,7 +2841,7 @@
         <v>1744.3333333333335</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>5</v>
       </c>
@@ -2890,7 +2890,7 @@
         <v>1994.6666666666667</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>6</v>
       </c>
@@ -2939,7 +2939,7 @@
         <v>2321</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>6</v>
       </c>
@@ -2988,7 +2988,7 @@
         <v>4768.666666666667</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>6</v>
       </c>
@@ -3037,7 +3037,7 @@
         <v>1928.6666666666665</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>6</v>
       </c>
@@ -3086,7 +3086,7 @@
         <v>2881</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>7</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>5348.3333333333339</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>7</v>
       </c>
@@ -3184,7 +3184,7 @@
         <v>1118.6666666666667</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>7</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>3556.666666666667</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>8</v>
       </c>
@@ -3282,7 +3282,7 @@
         <v>4884</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>8</v>
       </c>
@@ -3331,7 +3331,7 @@
         <v>3204</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>9</v>
       </c>
@@ -3380,7 +3380,7 @@
         <v>3091.3333333333335</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>1</v>
       </c>
@@ -3404,8 +3404,11 @@
       <c r="I47">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="N47" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2</v>
       </c>
@@ -3429,8 +3432,11 @@
       <c r="I48">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="N48" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>3</v>
       </c>
@@ -3454,8 +3460,11 @@
       <c r="I49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="N49" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>4</v>
       </c>
@@ -3479,8 +3488,11 @@
       <c r="I50">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="N50" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>5</v>
       </c>
@@ -3504,8 +3516,11 @@
       <c r="I51">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="N51" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>6</v>
       </c>
@@ -3527,8 +3542,11 @@
       <c r="I52">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="N52" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>7</v>
       </c>
@@ -3550,8 +3568,11 @@
       <c r="I53">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="N53" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>8</v>
       </c>
@@ -3573,8 +3594,11 @@
       <c r="I54">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="N54" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>9</v>
       </c>
@@ -3596,8 +3620,11 @@
       <c r="I55">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="N55" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>10</v>
       </c>
@@ -3617,6 +3644,9 @@
         <v>0</v>
       </c>
       <c r="I56">
+        <v>0</v>
+      </c>
+      <c r="N56" s="10">
         <v>0</v>
       </c>
     </row>

</xml_diff>